<commit_message>
Fix #### in the Excel workbook: pre-format dates and prices, widen columns
- dates written with a time part did not fit their column; the template now
  pre-formats data rows and format_sheet repairs filled workbooks
- 2 tests; README changelog

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/veri_toplama.xlsx
+++ b/data/templates/veri_toplama.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -65,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -74,6 +76,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -546,11 +550,11 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -672,6 +676,900 @@
           <t>sitede yazan</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="H3" s="4" t="n"/>
+    </row>
+    <row r="4">
+      <c r="H4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="H5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="H6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="H7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="H8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="H9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="H10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="H11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="H12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="H13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="H14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="H15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="H16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="H17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="H18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="H19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="H20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="H21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="H22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="H23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="H24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="H25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="H26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="H27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="H28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="H29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="H30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="H31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="H32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="H33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="H34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="H35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="H36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="H37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="H38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="H39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="H40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="H41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="H42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="H43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="H44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="H45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="H46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="H47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="H48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="H49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="H50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="H51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="H52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="H53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="H54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="H55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="H56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="H57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="H58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="H59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="H60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="H61" s="4" t="n"/>
+    </row>
+    <row r="62">
+      <c r="H62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="H63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="H64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="H65" s="4" t="n"/>
+    </row>
+    <row r="66">
+      <c r="H66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="H67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="H68" s="4" t="n"/>
+    </row>
+    <row r="69">
+      <c r="H69" s="4" t="n"/>
+    </row>
+    <row r="70">
+      <c r="H70" s="4" t="n"/>
+    </row>
+    <row r="71">
+      <c r="H71" s="4" t="n"/>
+    </row>
+    <row r="72">
+      <c r="H72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="H73" s="4" t="n"/>
+    </row>
+    <row r="74">
+      <c r="H74" s="4" t="n"/>
+    </row>
+    <row r="75">
+      <c r="H75" s="4" t="n"/>
+    </row>
+    <row r="76">
+      <c r="H76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="H77" s="4" t="n"/>
+    </row>
+    <row r="78">
+      <c r="H78" s="4" t="n"/>
+    </row>
+    <row r="79">
+      <c r="H79" s="4" t="n"/>
+    </row>
+    <row r="80">
+      <c r="H80" s="4" t="n"/>
+    </row>
+    <row r="81">
+      <c r="H81" s="4" t="n"/>
+    </row>
+    <row r="82">
+      <c r="H82" s="4" t="n"/>
+    </row>
+    <row r="83">
+      <c r="H83" s="4" t="n"/>
+    </row>
+    <row r="84">
+      <c r="H84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="H85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="H86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="H87" s="4" t="n"/>
+    </row>
+    <row r="88">
+      <c r="H88" s="4" t="n"/>
+    </row>
+    <row r="89">
+      <c r="H89" s="4" t="n"/>
+    </row>
+    <row r="90">
+      <c r="H90" s="4" t="n"/>
+    </row>
+    <row r="91">
+      <c r="H91" s="4" t="n"/>
+    </row>
+    <row r="92">
+      <c r="H92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="H93" s="4" t="n"/>
+    </row>
+    <row r="94">
+      <c r="H94" s="4" t="n"/>
+    </row>
+    <row r="95">
+      <c r="H95" s="4" t="n"/>
+    </row>
+    <row r="96">
+      <c r="H96" s="4" t="n"/>
+    </row>
+    <row r="97">
+      <c r="H97" s="4" t="n"/>
+    </row>
+    <row r="98">
+      <c r="H98" s="4" t="n"/>
+    </row>
+    <row r="99">
+      <c r="H99" s="4" t="n"/>
+    </row>
+    <row r="100">
+      <c r="H100" s="4" t="n"/>
+    </row>
+    <row r="101">
+      <c r="H101" s="4" t="n"/>
+    </row>
+    <row r="102">
+      <c r="H102" s="4" t="n"/>
+    </row>
+    <row r="103">
+      <c r="H103" s="4" t="n"/>
+    </row>
+    <row r="104">
+      <c r="H104" s="4" t="n"/>
+    </row>
+    <row r="105">
+      <c r="H105" s="4" t="n"/>
+    </row>
+    <row r="106">
+      <c r="H106" s="4" t="n"/>
+    </row>
+    <row r="107">
+      <c r="H107" s="4" t="n"/>
+    </row>
+    <row r="108">
+      <c r="H108" s="4" t="n"/>
+    </row>
+    <row r="109">
+      <c r="H109" s="4" t="n"/>
+    </row>
+    <row r="110">
+      <c r="H110" s="4" t="n"/>
+    </row>
+    <row r="111">
+      <c r="H111" s="4" t="n"/>
+    </row>
+    <row r="112">
+      <c r="H112" s="4" t="n"/>
+    </row>
+    <row r="113">
+      <c r="H113" s="4" t="n"/>
+    </row>
+    <row r="114">
+      <c r="H114" s="4" t="n"/>
+    </row>
+    <row r="115">
+      <c r="H115" s="4" t="n"/>
+    </row>
+    <row r="116">
+      <c r="H116" s="4" t="n"/>
+    </row>
+    <row r="117">
+      <c r="H117" s="4" t="n"/>
+    </row>
+    <row r="118">
+      <c r="H118" s="4" t="n"/>
+    </row>
+    <row r="119">
+      <c r="H119" s="4" t="n"/>
+    </row>
+    <row r="120">
+      <c r="H120" s="4" t="n"/>
+    </row>
+    <row r="121">
+      <c r="H121" s="4" t="n"/>
+    </row>
+    <row r="122">
+      <c r="H122" s="4" t="n"/>
+    </row>
+    <row r="123">
+      <c r="H123" s="4" t="n"/>
+    </row>
+    <row r="124">
+      <c r="H124" s="4" t="n"/>
+    </row>
+    <row r="125">
+      <c r="H125" s="4" t="n"/>
+    </row>
+    <row r="126">
+      <c r="H126" s="4" t="n"/>
+    </row>
+    <row r="127">
+      <c r="H127" s="4" t="n"/>
+    </row>
+    <row r="128">
+      <c r="H128" s="4" t="n"/>
+    </row>
+    <row r="129">
+      <c r="H129" s="4" t="n"/>
+    </row>
+    <row r="130">
+      <c r="H130" s="4" t="n"/>
+    </row>
+    <row r="131">
+      <c r="H131" s="4" t="n"/>
+    </row>
+    <row r="132">
+      <c r="H132" s="4" t="n"/>
+    </row>
+    <row r="133">
+      <c r="H133" s="4" t="n"/>
+    </row>
+    <row r="134">
+      <c r="H134" s="4" t="n"/>
+    </row>
+    <row r="135">
+      <c r="H135" s="4" t="n"/>
+    </row>
+    <row r="136">
+      <c r="H136" s="4" t="n"/>
+    </row>
+    <row r="137">
+      <c r="H137" s="4" t="n"/>
+    </row>
+    <row r="138">
+      <c r="H138" s="4" t="n"/>
+    </row>
+    <row r="139">
+      <c r="H139" s="4" t="n"/>
+    </row>
+    <row r="140">
+      <c r="H140" s="4" t="n"/>
+    </row>
+    <row r="141">
+      <c r="H141" s="4" t="n"/>
+    </row>
+    <row r="142">
+      <c r="H142" s="4" t="n"/>
+    </row>
+    <row r="143">
+      <c r="H143" s="4" t="n"/>
+    </row>
+    <row r="144">
+      <c r="H144" s="4" t="n"/>
+    </row>
+    <row r="145">
+      <c r="H145" s="4" t="n"/>
+    </row>
+    <row r="146">
+      <c r="H146" s="4" t="n"/>
+    </row>
+    <row r="147">
+      <c r="H147" s="4" t="n"/>
+    </row>
+    <row r="148">
+      <c r="H148" s="4" t="n"/>
+    </row>
+    <row r="149">
+      <c r="H149" s="4" t="n"/>
+    </row>
+    <row r="150">
+      <c r="H150" s="4" t="n"/>
+    </row>
+    <row r="151">
+      <c r="H151" s="4" t="n"/>
+    </row>
+    <row r="152">
+      <c r="H152" s="4" t="n"/>
+    </row>
+    <row r="153">
+      <c r="H153" s="4" t="n"/>
+    </row>
+    <row r="154">
+      <c r="H154" s="4" t="n"/>
+    </row>
+    <row r="155">
+      <c r="H155" s="4" t="n"/>
+    </row>
+    <row r="156">
+      <c r="H156" s="4" t="n"/>
+    </row>
+    <row r="157">
+      <c r="H157" s="4" t="n"/>
+    </row>
+    <row r="158">
+      <c r="H158" s="4" t="n"/>
+    </row>
+    <row r="159">
+      <c r="H159" s="4" t="n"/>
+    </row>
+    <row r="160">
+      <c r="H160" s="4" t="n"/>
+    </row>
+    <row r="161">
+      <c r="H161" s="4" t="n"/>
+    </row>
+    <row r="162">
+      <c r="H162" s="4" t="n"/>
+    </row>
+    <row r="163">
+      <c r="H163" s="4" t="n"/>
+    </row>
+    <row r="164">
+      <c r="H164" s="4" t="n"/>
+    </row>
+    <row r="165">
+      <c r="H165" s="4" t="n"/>
+    </row>
+    <row r="166">
+      <c r="H166" s="4" t="n"/>
+    </row>
+    <row r="167">
+      <c r="H167" s="4" t="n"/>
+    </row>
+    <row r="168">
+      <c r="H168" s="4" t="n"/>
+    </row>
+    <row r="169">
+      <c r="H169" s="4" t="n"/>
+    </row>
+    <row r="170">
+      <c r="H170" s="4" t="n"/>
+    </row>
+    <row r="171">
+      <c r="H171" s="4" t="n"/>
+    </row>
+    <row r="172">
+      <c r="H172" s="4" t="n"/>
+    </row>
+    <row r="173">
+      <c r="H173" s="4" t="n"/>
+    </row>
+    <row r="174">
+      <c r="H174" s="4" t="n"/>
+    </row>
+    <row r="175">
+      <c r="H175" s="4" t="n"/>
+    </row>
+    <row r="176">
+      <c r="H176" s="4" t="n"/>
+    </row>
+    <row r="177">
+      <c r="H177" s="4" t="n"/>
+    </row>
+    <row r="178">
+      <c r="H178" s="4" t="n"/>
+    </row>
+    <row r="179">
+      <c r="H179" s="4" t="n"/>
+    </row>
+    <row r="180">
+      <c r="H180" s="4" t="n"/>
+    </row>
+    <row r="181">
+      <c r="H181" s="4" t="n"/>
+    </row>
+    <row r="182">
+      <c r="H182" s="4" t="n"/>
+    </row>
+    <row r="183">
+      <c r="H183" s="4" t="n"/>
+    </row>
+    <row r="184">
+      <c r="H184" s="4" t="n"/>
+    </row>
+    <row r="185">
+      <c r="H185" s="4" t="n"/>
+    </row>
+    <row r="186">
+      <c r="H186" s="4" t="n"/>
+    </row>
+    <row r="187">
+      <c r="H187" s="4" t="n"/>
+    </row>
+    <row r="188">
+      <c r="H188" s="4" t="n"/>
+    </row>
+    <row r="189">
+      <c r="H189" s="4" t="n"/>
+    </row>
+    <row r="190">
+      <c r="H190" s="4" t="n"/>
+    </row>
+    <row r="191">
+      <c r="H191" s="4" t="n"/>
+    </row>
+    <row r="192">
+      <c r="H192" s="4" t="n"/>
+    </row>
+    <row r="193">
+      <c r="H193" s="4" t="n"/>
+    </row>
+    <row r="194">
+      <c r="H194" s="4" t="n"/>
+    </row>
+    <row r="195">
+      <c r="H195" s="4" t="n"/>
+    </row>
+    <row r="196">
+      <c r="H196" s="4" t="n"/>
+    </row>
+    <row r="197">
+      <c r="H197" s="4" t="n"/>
+    </row>
+    <row r="198">
+      <c r="H198" s="4" t="n"/>
+    </row>
+    <row r="199">
+      <c r="H199" s="4" t="n"/>
+    </row>
+    <row r="200">
+      <c r="H200" s="4" t="n"/>
+    </row>
+    <row r="201">
+      <c r="H201" s="4" t="n"/>
+    </row>
+    <row r="202">
+      <c r="H202" s="4" t="n"/>
+    </row>
+    <row r="203">
+      <c r="H203" s="4" t="n"/>
+    </row>
+    <row r="204">
+      <c r="H204" s="4" t="n"/>
+    </row>
+    <row r="205">
+      <c r="H205" s="4" t="n"/>
+    </row>
+    <row r="206">
+      <c r="H206" s="4" t="n"/>
+    </row>
+    <row r="207">
+      <c r="H207" s="4" t="n"/>
+    </row>
+    <row r="208">
+      <c r="H208" s="4" t="n"/>
+    </row>
+    <row r="209">
+      <c r="H209" s="4" t="n"/>
+    </row>
+    <row r="210">
+      <c r="H210" s="4" t="n"/>
+    </row>
+    <row r="211">
+      <c r="H211" s="4" t="n"/>
+    </row>
+    <row r="212">
+      <c r="H212" s="4" t="n"/>
+    </row>
+    <row r="213">
+      <c r="H213" s="4" t="n"/>
+    </row>
+    <row r="214">
+      <c r="H214" s="4" t="n"/>
+    </row>
+    <row r="215">
+      <c r="H215" s="4" t="n"/>
+    </row>
+    <row r="216">
+      <c r="H216" s="4" t="n"/>
+    </row>
+    <row r="217">
+      <c r="H217" s="4" t="n"/>
+    </row>
+    <row r="218">
+      <c r="H218" s="4" t="n"/>
+    </row>
+    <row r="219">
+      <c r="H219" s="4" t="n"/>
+    </row>
+    <row r="220">
+      <c r="H220" s="4" t="n"/>
+    </row>
+    <row r="221">
+      <c r="H221" s="4" t="n"/>
+    </row>
+    <row r="222">
+      <c r="H222" s="4" t="n"/>
+    </row>
+    <row r="223">
+      <c r="H223" s="4" t="n"/>
+    </row>
+    <row r="224">
+      <c r="H224" s="4" t="n"/>
+    </row>
+    <row r="225">
+      <c r="H225" s="4" t="n"/>
+    </row>
+    <row r="226">
+      <c r="H226" s="4" t="n"/>
+    </row>
+    <row r="227">
+      <c r="H227" s="4" t="n"/>
+    </row>
+    <row r="228">
+      <c r="H228" s="4" t="n"/>
+    </row>
+    <row r="229">
+      <c r="H229" s="4" t="n"/>
+    </row>
+    <row r="230">
+      <c r="H230" s="4" t="n"/>
+    </row>
+    <row r="231">
+      <c r="H231" s="4" t="n"/>
+    </row>
+    <row r="232">
+      <c r="H232" s="4" t="n"/>
+    </row>
+    <row r="233">
+      <c r="H233" s="4" t="n"/>
+    </row>
+    <row r="234">
+      <c r="H234" s="4" t="n"/>
+    </row>
+    <row r="235">
+      <c r="H235" s="4" t="n"/>
+    </row>
+    <row r="236">
+      <c r="H236" s="4" t="n"/>
+    </row>
+    <row r="237">
+      <c r="H237" s="4" t="n"/>
+    </row>
+    <row r="238">
+      <c r="H238" s="4" t="n"/>
+    </row>
+    <row r="239">
+      <c r="H239" s="4" t="n"/>
+    </row>
+    <row r="240">
+      <c r="H240" s="4" t="n"/>
+    </row>
+    <row r="241">
+      <c r="H241" s="4" t="n"/>
+    </row>
+    <row r="242">
+      <c r="H242" s="4" t="n"/>
+    </row>
+    <row r="243">
+      <c r="H243" s="4" t="n"/>
+    </row>
+    <row r="244">
+      <c r="H244" s="4" t="n"/>
+    </row>
+    <row r="245">
+      <c r="H245" s="4" t="n"/>
+    </row>
+    <row r="246">
+      <c r="H246" s="4" t="n"/>
+    </row>
+    <row r="247">
+      <c r="H247" s="4" t="n"/>
+    </row>
+    <row r="248">
+      <c r="H248" s="4" t="n"/>
+    </row>
+    <row r="249">
+      <c r="H249" s="4" t="n"/>
+    </row>
+    <row r="250">
+      <c r="H250" s="4" t="n"/>
+    </row>
+    <row r="251">
+      <c r="H251" s="4" t="n"/>
+    </row>
+    <row r="252">
+      <c r="H252" s="4" t="n"/>
+    </row>
+    <row r="253">
+      <c r="H253" s="4" t="n"/>
+    </row>
+    <row r="254">
+      <c r="H254" s="4" t="n"/>
+    </row>
+    <row r="255">
+      <c r="H255" s="4" t="n"/>
+    </row>
+    <row r="256">
+      <c r="H256" s="4" t="n"/>
+    </row>
+    <row r="257">
+      <c r="H257" s="4" t="n"/>
+    </row>
+    <row r="258">
+      <c r="H258" s="4" t="n"/>
+    </row>
+    <row r="259">
+      <c r="H259" s="4" t="n"/>
+    </row>
+    <row r="260">
+      <c r="H260" s="4" t="n"/>
+    </row>
+    <row r="261">
+      <c r="H261" s="4" t="n"/>
+    </row>
+    <row r="262">
+      <c r="H262" s="4" t="n"/>
+    </row>
+    <row r="263">
+      <c r="H263" s="4" t="n"/>
+    </row>
+    <row r="264">
+      <c r="H264" s="4" t="n"/>
+    </row>
+    <row r="265">
+      <c r="H265" s="4" t="n"/>
+    </row>
+    <row r="266">
+      <c r="H266" s="4" t="n"/>
+    </row>
+    <row r="267">
+      <c r="H267" s="4" t="n"/>
+    </row>
+    <row r="268">
+      <c r="H268" s="4" t="n"/>
+    </row>
+    <row r="269">
+      <c r="H269" s="4" t="n"/>
+    </row>
+    <row r="270">
+      <c r="H270" s="4" t="n"/>
+    </row>
+    <row r="271">
+      <c r="H271" s="4" t="n"/>
+    </row>
+    <row r="272">
+      <c r="H272" s="4" t="n"/>
+    </row>
+    <row r="273">
+      <c r="H273" s="4" t="n"/>
+    </row>
+    <row r="274">
+      <c r="H274" s="4" t="n"/>
+    </row>
+    <row r="275">
+      <c r="H275" s="4" t="n"/>
+    </row>
+    <row r="276">
+      <c r="H276" s="4" t="n"/>
+    </row>
+    <row r="277">
+      <c r="H277" s="4" t="n"/>
+    </row>
+    <row r="278">
+      <c r="H278" s="4" t="n"/>
+    </row>
+    <row r="279">
+      <c r="H279" s="4" t="n"/>
+    </row>
+    <row r="280">
+      <c r="H280" s="4" t="n"/>
+    </row>
+    <row r="281">
+      <c r="H281" s="4" t="n"/>
+    </row>
+    <row r="282">
+      <c r="H282" s="4" t="n"/>
+    </row>
+    <row r="283">
+      <c r="H283" s="4" t="n"/>
+    </row>
+    <row r="284">
+      <c r="H284" s="4" t="n"/>
+    </row>
+    <row r="285">
+      <c r="H285" s="4" t="n"/>
+    </row>
+    <row r="286">
+      <c r="H286" s="4" t="n"/>
+    </row>
+    <row r="287">
+      <c r="H287" s="4" t="n"/>
+    </row>
+    <row r="288">
+      <c r="H288" s="4" t="n"/>
+    </row>
+    <row r="289">
+      <c r="H289" s="4" t="n"/>
+    </row>
+    <row r="290">
+      <c r="H290" s="4" t="n"/>
+    </row>
+    <row r="291">
+      <c r="H291" s="4" t="n"/>
+    </row>
+    <row r="292">
+      <c r="H292" s="4" t="n"/>
+    </row>
+    <row r="293">
+      <c r="H293" s="4" t="n"/>
+    </row>
+    <row r="294">
+      <c r="H294" s="4" t="n"/>
+    </row>
+    <row r="295">
+      <c r="H295" s="4" t="n"/>
+    </row>
+    <row r="296">
+      <c r="H296" s="4" t="n"/>
+    </row>
+    <row r="297">
+      <c r="H297" s="4" t="n"/>
+    </row>
+    <row r="298">
+      <c r="H298" s="4" t="n"/>
+    </row>
+    <row r="299">
+      <c r="H299" s="4" t="n"/>
+    </row>
+    <row r="300">
+      <c r="H300" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -692,18 +1590,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -806,6 +1704,900 @@
           <t>sayfada yazan etiket adı</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="I3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="I4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="I5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="I6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="I7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="I8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="I9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="I10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="I11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="I12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="I13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="I14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="I15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="I16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="I17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="I18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="I19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="I20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="I21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="I22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="I23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="I24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="I25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="I26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="I27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="I28" s="5" t="n"/>
+    </row>
+    <row r="29">
+      <c r="I29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="I30" s="5" t="n"/>
+    </row>
+    <row r="31">
+      <c r="I31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="I32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="I33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="I34" s="5" t="n"/>
+    </row>
+    <row r="35">
+      <c r="I35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="I36" s="5" t="n"/>
+    </row>
+    <row r="37">
+      <c r="I37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="I38" s="5" t="n"/>
+    </row>
+    <row r="39">
+      <c r="I39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="I40" s="5" t="n"/>
+    </row>
+    <row r="41">
+      <c r="I41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="I42" s="5" t="n"/>
+    </row>
+    <row r="43">
+      <c r="I43" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="I44" s="5" t="n"/>
+    </row>
+    <row r="45">
+      <c r="I45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="I46" s="5" t="n"/>
+    </row>
+    <row r="47">
+      <c r="I47" s="5" t="n"/>
+    </row>
+    <row r="48">
+      <c r="I48" s="5" t="n"/>
+    </row>
+    <row r="49">
+      <c r="I49" s="5" t="n"/>
+    </row>
+    <row r="50">
+      <c r="I50" s="5" t="n"/>
+    </row>
+    <row r="51">
+      <c r="I51" s="5" t="n"/>
+    </row>
+    <row r="52">
+      <c r="I52" s="5" t="n"/>
+    </row>
+    <row r="53">
+      <c r="I53" s="5" t="n"/>
+    </row>
+    <row r="54">
+      <c r="I54" s="5" t="n"/>
+    </row>
+    <row r="55">
+      <c r="I55" s="5" t="n"/>
+    </row>
+    <row r="56">
+      <c r="I56" s="5" t="n"/>
+    </row>
+    <row r="57">
+      <c r="I57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="I58" s="5" t="n"/>
+    </row>
+    <row r="59">
+      <c r="I59" s="5" t="n"/>
+    </row>
+    <row r="60">
+      <c r="I60" s="5" t="n"/>
+    </row>
+    <row r="61">
+      <c r="I61" s="5" t="n"/>
+    </row>
+    <row r="62">
+      <c r="I62" s="5" t="n"/>
+    </row>
+    <row r="63">
+      <c r="I63" s="5" t="n"/>
+    </row>
+    <row r="64">
+      <c r="I64" s="5" t="n"/>
+    </row>
+    <row r="65">
+      <c r="I65" s="5" t="n"/>
+    </row>
+    <row r="66">
+      <c r="I66" s="5" t="n"/>
+    </row>
+    <row r="67">
+      <c r="I67" s="5" t="n"/>
+    </row>
+    <row r="68">
+      <c r="I68" s="5" t="n"/>
+    </row>
+    <row r="69">
+      <c r="I69" s="5" t="n"/>
+    </row>
+    <row r="70">
+      <c r="I70" s="5" t="n"/>
+    </row>
+    <row r="71">
+      <c r="I71" s="5" t="n"/>
+    </row>
+    <row r="72">
+      <c r="I72" s="5" t="n"/>
+    </row>
+    <row r="73">
+      <c r="I73" s="5" t="n"/>
+    </row>
+    <row r="74">
+      <c r="I74" s="5" t="n"/>
+    </row>
+    <row r="75">
+      <c r="I75" s="5" t="n"/>
+    </row>
+    <row r="76">
+      <c r="I76" s="5" t="n"/>
+    </row>
+    <row r="77">
+      <c r="I77" s="5" t="n"/>
+    </row>
+    <row r="78">
+      <c r="I78" s="5" t="n"/>
+    </row>
+    <row r="79">
+      <c r="I79" s="5" t="n"/>
+    </row>
+    <row r="80">
+      <c r="I80" s="5" t="n"/>
+    </row>
+    <row r="81">
+      <c r="I81" s="5" t="n"/>
+    </row>
+    <row r="82">
+      <c r="I82" s="5" t="n"/>
+    </row>
+    <row r="83">
+      <c r="I83" s="5" t="n"/>
+    </row>
+    <row r="84">
+      <c r="I84" s="5" t="n"/>
+    </row>
+    <row r="85">
+      <c r="I85" s="5" t="n"/>
+    </row>
+    <row r="86">
+      <c r="I86" s="5" t="n"/>
+    </row>
+    <row r="87">
+      <c r="I87" s="5" t="n"/>
+    </row>
+    <row r="88">
+      <c r="I88" s="5" t="n"/>
+    </row>
+    <row r="89">
+      <c r="I89" s="5" t="n"/>
+    </row>
+    <row r="90">
+      <c r="I90" s="5" t="n"/>
+    </row>
+    <row r="91">
+      <c r="I91" s="5" t="n"/>
+    </row>
+    <row r="92">
+      <c r="I92" s="5" t="n"/>
+    </row>
+    <row r="93">
+      <c r="I93" s="5" t="n"/>
+    </row>
+    <row r="94">
+      <c r="I94" s="5" t="n"/>
+    </row>
+    <row r="95">
+      <c r="I95" s="5" t="n"/>
+    </row>
+    <row r="96">
+      <c r="I96" s="5" t="n"/>
+    </row>
+    <row r="97">
+      <c r="I97" s="5" t="n"/>
+    </row>
+    <row r="98">
+      <c r="I98" s="5" t="n"/>
+    </row>
+    <row r="99">
+      <c r="I99" s="5" t="n"/>
+    </row>
+    <row r="100">
+      <c r="I100" s="5" t="n"/>
+    </row>
+    <row r="101">
+      <c r="I101" s="5" t="n"/>
+    </row>
+    <row r="102">
+      <c r="I102" s="5" t="n"/>
+    </row>
+    <row r="103">
+      <c r="I103" s="5" t="n"/>
+    </row>
+    <row r="104">
+      <c r="I104" s="5" t="n"/>
+    </row>
+    <row r="105">
+      <c r="I105" s="5" t="n"/>
+    </row>
+    <row r="106">
+      <c r="I106" s="5" t="n"/>
+    </row>
+    <row r="107">
+      <c r="I107" s="5" t="n"/>
+    </row>
+    <row r="108">
+      <c r="I108" s="5" t="n"/>
+    </row>
+    <row r="109">
+      <c r="I109" s="5" t="n"/>
+    </row>
+    <row r="110">
+      <c r="I110" s="5" t="n"/>
+    </row>
+    <row r="111">
+      <c r="I111" s="5" t="n"/>
+    </row>
+    <row r="112">
+      <c r="I112" s="5" t="n"/>
+    </row>
+    <row r="113">
+      <c r="I113" s="5" t="n"/>
+    </row>
+    <row r="114">
+      <c r="I114" s="5" t="n"/>
+    </row>
+    <row r="115">
+      <c r="I115" s="5" t="n"/>
+    </row>
+    <row r="116">
+      <c r="I116" s="5" t="n"/>
+    </row>
+    <row r="117">
+      <c r="I117" s="5" t="n"/>
+    </row>
+    <row r="118">
+      <c r="I118" s="5" t="n"/>
+    </row>
+    <row r="119">
+      <c r="I119" s="5" t="n"/>
+    </row>
+    <row r="120">
+      <c r="I120" s="5" t="n"/>
+    </row>
+    <row r="121">
+      <c r="I121" s="5" t="n"/>
+    </row>
+    <row r="122">
+      <c r="I122" s="5" t="n"/>
+    </row>
+    <row r="123">
+      <c r="I123" s="5" t="n"/>
+    </row>
+    <row r="124">
+      <c r="I124" s="5" t="n"/>
+    </row>
+    <row r="125">
+      <c r="I125" s="5" t="n"/>
+    </row>
+    <row r="126">
+      <c r="I126" s="5" t="n"/>
+    </row>
+    <row r="127">
+      <c r="I127" s="5" t="n"/>
+    </row>
+    <row r="128">
+      <c r="I128" s="5" t="n"/>
+    </row>
+    <row r="129">
+      <c r="I129" s="5" t="n"/>
+    </row>
+    <row r="130">
+      <c r="I130" s="5" t="n"/>
+    </row>
+    <row r="131">
+      <c r="I131" s="5" t="n"/>
+    </row>
+    <row r="132">
+      <c r="I132" s="5" t="n"/>
+    </row>
+    <row r="133">
+      <c r="I133" s="5" t="n"/>
+    </row>
+    <row r="134">
+      <c r="I134" s="5" t="n"/>
+    </row>
+    <row r="135">
+      <c r="I135" s="5" t="n"/>
+    </row>
+    <row r="136">
+      <c r="I136" s="5" t="n"/>
+    </row>
+    <row r="137">
+      <c r="I137" s="5" t="n"/>
+    </row>
+    <row r="138">
+      <c r="I138" s="5" t="n"/>
+    </row>
+    <row r="139">
+      <c r="I139" s="5" t="n"/>
+    </row>
+    <row r="140">
+      <c r="I140" s="5" t="n"/>
+    </row>
+    <row r="141">
+      <c r="I141" s="5" t="n"/>
+    </row>
+    <row r="142">
+      <c r="I142" s="5" t="n"/>
+    </row>
+    <row r="143">
+      <c r="I143" s="5" t="n"/>
+    </row>
+    <row r="144">
+      <c r="I144" s="5" t="n"/>
+    </row>
+    <row r="145">
+      <c r="I145" s="5" t="n"/>
+    </row>
+    <row r="146">
+      <c r="I146" s="5" t="n"/>
+    </row>
+    <row r="147">
+      <c r="I147" s="5" t="n"/>
+    </row>
+    <row r="148">
+      <c r="I148" s="5" t="n"/>
+    </row>
+    <row r="149">
+      <c r="I149" s="5" t="n"/>
+    </row>
+    <row r="150">
+      <c r="I150" s="5" t="n"/>
+    </row>
+    <row r="151">
+      <c r="I151" s="5" t="n"/>
+    </row>
+    <row r="152">
+      <c r="I152" s="5" t="n"/>
+    </row>
+    <row r="153">
+      <c r="I153" s="5" t="n"/>
+    </row>
+    <row r="154">
+      <c r="I154" s="5" t="n"/>
+    </row>
+    <row r="155">
+      <c r="I155" s="5" t="n"/>
+    </row>
+    <row r="156">
+      <c r="I156" s="5" t="n"/>
+    </row>
+    <row r="157">
+      <c r="I157" s="5" t="n"/>
+    </row>
+    <row r="158">
+      <c r="I158" s="5" t="n"/>
+    </row>
+    <row r="159">
+      <c r="I159" s="5" t="n"/>
+    </row>
+    <row r="160">
+      <c r="I160" s="5" t="n"/>
+    </row>
+    <row r="161">
+      <c r="I161" s="5" t="n"/>
+    </row>
+    <row r="162">
+      <c r="I162" s="5" t="n"/>
+    </row>
+    <row r="163">
+      <c r="I163" s="5" t="n"/>
+    </row>
+    <row r="164">
+      <c r="I164" s="5" t="n"/>
+    </row>
+    <row r="165">
+      <c r="I165" s="5" t="n"/>
+    </row>
+    <row r="166">
+      <c r="I166" s="5" t="n"/>
+    </row>
+    <row r="167">
+      <c r="I167" s="5" t="n"/>
+    </row>
+    <row r="168">
+      <c r="I168" s="5" t="n"/>
+    </row>
+    <row r="169">
+      <c r="I169" s="5" t="n"/>
+    </row>
+    <row r="170">
+      <c r="I170" s="5" t="n"/>
+    </row>
+    <row r="171">
+      <c r="I171" s="5" t="n"/>
+    </row>
+    <row r="172">
+      <c r="I172" s="5" t="n"/>
+    </row>
+    <row r="173">
+      <c r="I173" s="5" t="n"/>
+    </row>
+    <row r="174">
+      <c r="I174" s="5" t="n"/>
+    </row>
+    <row r="175">
+      <c r="I175" s="5" t="n"/>
+    </row>
+    <row r="176">
+      <c r="I176" s="5" t="n"/>
+    </row>
+    <row r="177">
+      <c r="I177" s="5" t="n"/>
+    </row>
+    <row r="178">
+      <c r="I178" s="5" t="n"/>
+    </row>
+    <row r="179">
+      <c r="I179" s="5" t="n"/>
+    </row>
+    <row r="180">
+      <c r="I180" s="5" t="n"/>
+    </row>
+    <row r="181">
+      <c r="I181" s="5" t="n"/>
+    </row>
+    <row r="182">
+      <c r="I182" s="5" t="n"/>
+    </row>
+    <row r="183">
+      <c r="I183" s="5" t="n"/>
+    </row>
+    <row r="184">
+      <c r="I184" s="5" t="n"/>
+    </row>
+    <row r="185">
+      <c r="I185" s="5" t="n"/>
+    </row>
+    <row r="186">
+      <c r="I186" s="5" t="n"/>
+    </row>
+    <row r="187">
+      <c r="I187" s="5" t="n"/>
+    </row>
+    <row r="188">
+      <c r="I188" s="5" t="n"/>
+    </row>
+    <row r="189">
+      <c r="I189" s="5" t="n"/>
+    </row>
+    <row r="190">
+      <c r="I190" s="5" t="n"/>
+    </row>
+    <row r="191">
+      <c r="I191" s="5" t="n"/>
+    </row>
+    <row r="192">
+      <c r="I192" s="5" t="n"/>
+    </row>
+    <row r="193">
+      <c r="I193" s="5" t="n"/>
+    </row>
+    <row r="194">
+      <c r="I194" s="5" t="n"/>
+    </row>
+    <row r="195">
+      <c r="I195" s="5" t="n"/>
+    </row>
+    <row r="196">
+      <c r="I196" s="5" t="n"/>
+    </row>
+    <row r="197">
+      <c r="I197" s="5" t="n"/>
+    </row>
+    <row r="198">
+      <c r="I198" s="5" t="n"/>
+    </row>
+    <row r="199">
+      <c r="I199" s="5" t="n"/>
+    </row>
+    <row r="200">
+      <c r="I200" s="5" t="n"/>
+    </row>
+    <row r="201">
+      <c r="I201" s="5" t="n"/>
+    </row>
+    <row r="202">
+      <c r="I202" s="5" t="n"/>
+    </row>
+    <row r="203">
+      <c r="I203" s="5" t="n"/>
+    </row>
+    <row r="204">
+      <c r="I204" s="5" t="n"/>
+    </row>
+    <row r="205">
+      <c r="I205" s="5" t="n"/>
+    </row>
+    <row r="206">
+      <c r="I206" s="5" t="n"/>
+    </row>
+    <row r="207">
+      <c r="I207" s="5" t="n"/>
+    </row>
+    <row r="208">
+      <c r="I208" s="5" t="n"/>
+    </row>
+    <row r="209">
+      <c r="I209" s="5" t="n"/>
+    </row>
+    <row r="210">
+      <c r="I210" s="5" t="n"/>
+    </row>
+    <row r="211">
+      <c r="I211" s="5" t="n"/>
+    </row>
+    <row r="212">
+      <c r="I212" s="5" t="n"/>
+    </row>
+    <row r="213">
+      <c r="I213" s="5" t="n"/>
+    </row>
+    <row r="214">
+      <c r="I214" s="5" t="n"/>
+    </row>
+    <row r="215">
+      <c r="I215" s="5" t="n"/>
+    </row>
+    <row r="216">
+      <c r="I216" s="5" t="n"/>
+    </row>
+    <row r="217">
+      <c r="I217" s="5" t="n"/>
+    </row>
+    <row r="218">
+      <c r="I218" s="5" t="n"/>
+    </row>
+    <row r="219">
+      <c r="I219" s="5" t="n"/>
+    </row>
+    <row r="220">
+      <c r="I220" s="5" t="n"/>
+    </row>
+    <row r="221">
+      <c r="I221" s="5" t="n"/>
+    </row>
+    <row r="222">
+      <c r="I222" s="5" t="n"/>
+    </row>
+    <row r="223">
+      <c r="I223" s="5" t="n"/>
+    </row>
+    <row r="224">
+      <c r="I224" s="5" t="n"/>
+    </row>
+    <row r="225">
+      <c r="I225" s="5" t="n"/>
+    </row>
+    <row r="226">
+      <c r="I226" s="5" t="n"/>
+    </row>
+    <row r="227">
+      <c r="I227" s="5" t="n"/>
+    </row>
+    <row r="228">
+      <c r="I228" s="5" t="n"/>
+    </row>
+    <row r="229">
+      <c r="I229" s="5" t="n"/>
+    </row>
+    <row r="230">
+      <c r="I230" s="5" t="n"/>
+    </row>
+    <row r="231">
+      <c r="I231" s="5" t="n"/>
+    </row>
+    <row r="232">
+      <c r="I232" s="5" t="n"/>
+    </row>
+    <row r="233">
+      <c r="I233" s="5" t="n"/>
+    </row>
+    <row r="234">
+      <c r="I234" s="5" t="n"/>
+    </row>
+    <row r="235">
+      <c r="I235" s="5" t="n"/>
+    </row>
+    <row r="236">
+      <c r="I236" s="5" t="n"/>
+    </row>
+    <row r="237">
+      <c r="I237" s="5" t="n"/>
+    </row>
+    <row r="238">
+      <c r="I238" s="5" t="n"/>
+    </row>
+    <row r="239">
+      <c r="I239" s="5" t="n"/>
+    </row>
+    <row r="240">
+      <c r="I240" s="5" t="n"/>
+    </row>
+    <row r="241">
+      <c r="I241" s="5" t="n"/>
+    </row>
+    <row r="242">
+      <c r="I242" s="5" t="n"/>
+    </row>
+    <row r="243">
+      <c r="I243" s="5" t="n"/>
+    </row>
+    <row r="244">
+      <c r="I244" s="5" t="n"/>
+    </row>
+    <row r="245">
+      <c r="I245" s="5" t="n"/>
+    </row>
+    <row r="246">
+      <c r="I246" s="5" t="n"/>
+    </row>
+    <row r="247">
+      <c r="I247" s="5" t="n"/>
+    </row>
+    <row r="248">
+      <c r="I248" s="5" t="n"/>
+    </row>
+    <row r="249">
+      <c r="I249" s="5" t="n"/>
+    </row>
+    <row r="250">
+      <c r="I250" s="5" t="n"/>
+    </row>
+    <row r="251">
+      <c r="I251" s="5" t="n"/>
+    </row>
+    <row r="252">
+      <c r="I252" s="5" t="n"/>
+    </row>
+    <row r="253">
+      <c r="I253" s="5" t="n"/>
+    </row>
+    <row r="254">
+      <c r="I254" s="5" t="n"/>
+    </row>
+    <row r="255">
+      <c r="I255" s="5" t="n"/>
+    </row>
+    <row r="256">
+      <c r="I256" s="5" t="n"/>
+    </row>
+    <row r="257">
+      <c r="I257" s="5" t="n"/>
+    </row>
+    <row r="258">
+      <c r="I258" s="5" t="n"/>
+    </row>
+    <row r="259">
+      <c r="I259" s="5" t="n"/>
+    </row>
+    <row r="260">
+      <c r="I260" s="5" t="n"/>
+    </row>
+    <row r="261">
+      <c r="I261" s="5" t="n"/>
+    </row>
+    <row r="262">
+      <c r="I262" s="5" t="n"/>
+    </row>
+    <row r="263">
+      <c r="I263" s="5" t="n"/>
+    </row>
+    <row r="264">
+      <c r="I264" s="5" t="n"/>
+    </row>
+    <row r="265">
+      <c r="I265" s="5" t="n"/>
+    </row>
+    <row r="266">
+      <c r="I266" s="5" t="n"/>
+    </row>
+    <row r="267">
+      <c r="I267" s="5" t="n"/>
+    </row>
+    <row r="268">
+      <c r="I268" s="5" t="n"/>
+    </row>
+    <row r="269">
+      <c r="I269" s="5" t="n"/>
+    </row>
+    <row r="270">
+      <c r="I270" s="5" t="n"/>
+    </row>
+    <row r="271">
+      <c r="I271" s="5" t="n"/>
+    </row>
+    <row r="272">
+      <c r="I272" s="5" t="n"/>
+    </row>
+    <row r="273">
+      <c r="I273" s="5" t="n"/>
+    </row>
+    <row r="274">
+      <c r="I274" s="5" t="n"/>
+    </row>
+    <row r="275">
+      <c r="I275" s="5" t="n"/>
+    </row>
+    <row r="276">
+      <c r="I276" s="5" t="n"/>
+    </row>
+    <row r="277">
+      <c r="I277" s="5" t="n"/>
+    </row>
+    <row r="278">
+      <c r="I278" s="5" t="n"/>
+    </row>
+    <row r="279">
+      <c r="I279" s="5" t="n"/>
+    </row>
+    <row r="280">
+      <c r="I280" s="5" t="n"/>
+    </row>
+    <row r="281">
+      <c r="I281" s="5" t="n"/>
+    </row>
+    <row r="282">
+      <c r="I282" s="5" t="n"/>
+    </row>
+    <row r="283">
+      <c r="I283" s="5" t="n"/>
+    </row>
+    <row r="284">
+      <c r="I284" s="5" t="n"/>
+    </row>
+    <row r="285">
+      <c r="I285" s="5" t="n"/>
+    </row>
+    <row r="286">
+      <c r="I286" s="5" t="n"/>
+    </row>
+    <row r="287">
+      <c r="I287" s="5" t="n"/>
+    </row>
+    <row r="288">
+      <c r="I288" s="5" t="n"/>
+    </row>
+    <row r="289">
+      <c r="I289" s="5" t="n"/>
+    </row>
+    <row r="290">
+      <c r="I290" s="5" t="n"/>
+    </row>
+    <row r="291">
+      <c r="I291" s="5" t="n"/>
+    </row>
+    <row r="292">
+      <c r="I292" s="5" t="n"/>
+    </row>
+    <row r="293">
+      <c r="I293" s="5" t="n"/>
+    </row>
+    <row r="294">
+      <c r="I294" s="5" t="n"/>
+    </row>
+    <row r="295">
+      <c r="I295" s="5" t="n"/>
+    </row>
+    <row r="296">
+      <c r="I296" s="5" t="n"/>
+    </row>
+    <row r="297">
+      <c r="I297" s="5" t="n"/>
+    </row>
+    <row r="298">
+      <c r="I298" s="5" t="n"/>
+    </row>
+    <row r="299">
+      <c r="I299" s="5" t="n"/>
+    </row>
+    <row r="300">
+      <c r="I300" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>